<commit_message>
Fix alignment indent setter
The IXLAlignment.Indent setter should also update reading order,
because Indent must be used along with Left,Right or Distributed
alignments. Excel will discard the Indent value with other horizontal
alignments.

This setter logic is the original behavior (with
InvalidOperationException instead, because problem is not the argument,
but the current state).

The StyleAlignment test file has been updated updated with the new
style writer, no semantic change.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Styles/StyleAlignment.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Styles/StyleAlignment.xlsx
@@ -49,97 +49,80 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="10">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="2" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="1" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="2" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="45" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="255" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment justifyLastLine="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment relativeIndent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="45"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -449,37 +432,37 @@
       </x:c>
     </x:row>
     <x:row r="5" spans="1:2">
-      <x:c r="B5" s="0" t="s">
+      <x:c r="B5" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:2">
-      <x:c r="B6" s="4" t="s">
+      <x:c r="B6" s="5" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:2">
-      <x:c r="B7" s="5" t="s">
+      <x:c r="B7" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:2">
-      <x:c r="B8" s="6" t="s">
+      <x:c r="B8" s="7" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:2">
-      <x:c r="B9" s="7" t="s">
+      <x:c r="B9" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:2">
-      <x:c r="B10" s="8" t="s">
+      <x:c r="B10" s="9" t="s">
         <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:2">
-      <x:c r="B11" s="9" t="s">
+      <x:c r="B11" s="10" t="s">
         <x:v>9</x:v>
       </x:c>
     </x:row>

</xml_diff>